<commit_message>
Update execution timestamps in evaluation notebook for consistency
</commit_message>
<xml_diff>
--- a/data/output/rda/RDA_simple14_revised.xlsx
+++ b/data/output/rda/RDA_simple14_revised.xlsx
@@ -295,7 +295,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -471,6 +471,21 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -830,57 +845,57 @@
     </row>
     <row r="2">
       <c r="A2" s="55" t="n"/>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="69" t="inlineStr">
         <is>
           <t>Item 1</t>
         </is>
       </c>
-      <c r="C2" s="16" t="inlineStr">
+      <c r="C2" s="69" t="inlineStr">
         <is>
           <t>Item 2</t>
         </is>
       </c>
-      <c r="D2" s="16" t="inlineStr">
+      <c r="D2" s="69" t="inlineStr">
         <is>
           <t>Item 3</t>
         </is>
       </c>
-      <c r="E2" s="16" t="inlineStr">
+      <c r="E2" s="69" t="inlineStr">
         <is>
           <t>Item 4</t>
         </is>
       </c>
-      <c r="F2" s="16" t="inlineStr">
+      <c r="F2" s="69" t="inlineStr">
         <is>
           <t>Item 5</t>
         </is>
       </c>
-      <c r="G2" s="16" t="inlineStr">
+      <c r="G2" s="69" t="inlineStr">
         <is>
           <t>Item 6</t>
         </is>
       </c>
-      <c r="H2" s="16" t="inlineStr">
+      <c r="H2" s="69" t="inlineStr">
         <is>
           <t>Item 7</t>
         </is>
       </c>
-      <c r="I2" s="16" t="inlineStr">
+      <c r="I2" s="69" t="inlineStr">
         <is>
           <t>Item 8</t>
         </is>
       </c>
-      <c r="J2" s="16" t="inlineStr">
+      <c r="J2" s="69" t="inlineStr">
         <is>
           <t>Item 9</t>
         </is>
       </c>
-      <c r="K2" s="16" t="inlineStr">
+      <c r="K2" s="69" t="inlineStr">
         <is>
           <t>Item 10</t>
         </is>
       </c>
-      <c r="L2" s="16" t="inlineStr">
+      <c r="L2" s="69" t="inlineStr">
         <is>
           <t>Item 11</t>
         </is>
@@ -888,7 +903,7 @@
       <c r="M2" s="14" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>$</t>
         </is>
@@ -907,7 +922,7 @@
       <c r="M3" s="14" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>dmp</t>
         </is>
@@ -926,12 +941,12 @@
       <c r="M4" s="14" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>dmp.title</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr">
+      <c r="B5" s="70" t="inlineStr">
         <is>
           <t>Hakai Institute Juvenile Salmon Program Time Series</t>
         </is>
@@ -949,7 +964,7 @@
       <c r="M5" s="14" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>dmp.description</t>
         </is>
@@ -968,7 +983,7 @@
       <c r="M6" s="14" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>dmp.dmp_id</t>
         </is>
@@ -987,12 +1002,12 @@
       <c r="M7" s="14" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>dmp.dmp_id.identifier</t>
         </is>
       </c>
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="70" t="inlineStr">
         <is>
           <t>https://doi.org/10.48321/D1CW23</t>
         </is>
@@ -1010,12 +1025,16 @@
       <c r="M8" s="14" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>dmp.dmp_id.type</t>
         </is>
       </c>
-      <c r="B9" s="28" t="n"/>
+      <c r="B9" s="71" t="inlineStr">
+        <is>
+          <t>doi</t>
+        </is>
+      </c>
       <c r="C9" s="22" t="n"/>
       <c r="D9" s="22" t="n"/>
       <c r="E9" s="22" t="n"/>
@@ -1029,12 +1048,16 @@
       <c r="M9" s="14" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>dmp.created</t>
         </is>
       </c>
-      <c r="B10" s="28" t="n"/>
+      <c r="B10" s="71" t="inlineStr">
+        <is>
+          <t>2015-05-12T00:00:00Z</t>
+        </is>
+      </c>
       <c r="C10" s="22" t="n"/>
       <c r="D10" s="22" t="n"/>
       <c r="E10" s="22" t="n"/>
@@ -1048,12 +1071,12 @@
       <c r="M10" s="14" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>dmp.modified</t>
         </is>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B11" s="70" t="inlineStr">
         <is>
           <t>2024-06-11T00:00:00Z</t>
         </is>
@@ -1071,12 +1094,12 @@
       <c r="M11" s="14" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>dmp.ethical_issues_exist</t>
         </is>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1094,7 +1117,7 @@
       <c r="M12" s="14" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>dmp.ethical_issues_description</t>
         </is>
@@ -1113,7 +1136,7 @@
       <c r="M13" s="14" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>dmp.ethical_issues_report</t>
         </is>
@@ -1132,12 +1155,16 @@
       <c r="M14" s="14" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>dmp.language</t>
         </is>
       </c>
-      <c r="B15" s="22" t="n"/>
+      <c r="B15" s="70" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
       <c r="C15" s="22" t="n"/>
       <c r="D15" s="22" t="n"/>
       <c r="E15" s="22" t="n"/>
@@ -1151,7 +1178,7 @@
       <c r="M15" s="14" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>dmp.contact</t>
         </is>
@@ -1175,7 +1202,7 @@
           <t>dmp.contact.name</t>
         </is>
       </c>
-      <c r="B17" s="22" t="inlineStr">
+      <c r="B17" s="70" t="inlineStr">
         <is>
           <t>Brett Johnson</t>
         </is>
@@ -1193,7 +1220,7 @@
       <c r="M17" s="14" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>dmp.contact.mbox</t>
         </is>
@@ -1212,7 +1239,7 @@
       <c r="M18" s="14" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>dmp.contact.affiliation</t>
         </is>
@@ -1231,7 +1258,7 @@
       <c r="M19" s="14" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>dmp.contact.affiliation[]</t>
         </is>
@@ -1250,12 +1277,12 @@
       <c r="M20" s="14" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>dmp.contact.affiliation[].name</t>
         </is>
       </c>
-      <c r="B21" s="22" t="inlineStr">
+      <c r="B21" s="70" t="inlineStr">
         <is>
           <t>Hakai Institute</t>
         </is>
@@ -1273,7 +1300,7 @@
       <c r="M21" s="14" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>dmp.contact.affiliation[].affiliation_id</t>
         </is>
@@ -1292,7 +1319,7 @@
       <c r="M22" s="14" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>dmp.contact.affiliation[].affiliation_id.identifier</t>
         </is>
@@ -1311,7 +1338,7 @@
       <c r="M23" s="14" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="22" t="inlineStr">
         <is>
           <t>dmp.contact.affiliation[].affiliation_id.type</t>
         </is>
@@ -1330,7 +1357,7 @@
       <c r="M24" s="14" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="18" t="inlineStr">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>dmp.contact.contact_id</t>
         </is>
@@ -1349,7 +1376,7 @@
       <c r="M25" s="14" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="18" t="inlineStr">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>dmp.contact.contact_id[]</t>
         </is>
@@ -1368,12 +1395,12 @@
       <c r="M26" s="14" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="18" t="inlineStr">
+      <c r="A27" s="22" t="inlineStr">
         <is>
           <t>dmp.contact.contact_id[].identifier</t>
         </is>
       </c>
-      <c r="B27" s="22" t="inlineStr">
+      <c r="B27" s="70" t="inlineStr">
         <is>
           <t>0000-0001-9317-0364</t>
         </is>
@@ -1391,12 +1418,12 @@
       <c r="M27" s="14" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="18" t="inlineStr">
+      <c r="A28" s="22" t="inlineStr">
         <is>
           <t>dmp.contact.contact_id[].type</t>
         </is>
       </c>
-      <c r="B28" s="22" t="inlineStr">
+      <c r="B28" s="70" t="inlineStr">
         <is>
           <t>orcid</t>
         </is>
@@ -1414,7 +1441,7 @@
       <c r="M28" s="14" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="18" t="inlineStr">
+      <c r="A29" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor</t>
         </is>
@@ -1433,7 +1460,7 @@
       <c r="M29" s="14" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="inlineStr">
+      <c r="A30" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor[]</t>
         </is>
@@ -1452,27 +1479,27 @@
       <c r="M30" s="14" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="18" t="inlineStr">
+      <c r="A31" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor[].name</t>
         </is>
       </c>
-      <c r="B31" s="22" t="inlineStr">
+      <c r="B31" s="70" t="inlineStr">
         <is>
           <t>Brett Johnson</t>
         </is>
       </c>
-      <c r="C31" s="22" t="inlineStr">
+      <c r="C31" s="70" t="inlineStr">
         <is>
           <t>Brian Hunt</t>
         </is>
       </c>
-      <c r="D31" s="22" t="inlineStr">
+      <c r="D31" s="70" t="inlineStr">
         <is>
           <t>Tim van der Stap</t>
         </is>
       </c>
-      <c r="E31" s="22" t="inlineStr">
+      <c r="E31" s="70" t="inlineStr">
         <is>
           <t>Krystal Bachen</t>
         </is>
@@ -1487,7 +1514,7 @@
       <c r="M31" s="14" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="18" t="inlineStr">
+      <c r="A32" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor[].contributor_id</t>
         </is>
@@ -1506,7 +1533,7 @@
       <c r="M32" s="14" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="18" t="inlineStr">
+      <c r="A33" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor[].contributor_id[]</t>
         </is>
@@ -1525,7 +1552,7 @@
       <c r="M33" s="14" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="inlineStr">
+      <c r="A34" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor[].contributor_id[].identifier</t>
         </is>
@@ -1544,7 +1571,7 @@
       <c r="M34" s="14" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="inlineStr">
+      <c r="A35" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor[].contributor_id[].type</t>
         </is>
@@ -1563,7 +1590,7 @@
       <c r="M35" s="14" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="inlineStr">
+      <c r="A36" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor[].affiliation</t>
         </is>
@@ -1582,7 +1609,7 @@
       <c r="M36" s="14" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="18" t="inlineStr">
+      <c r="A37" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor[].affiliation[]</t>
         </is>
@@ -1601,7 +1628,7 @@
       <c r="M37" s="14" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="18" t="inlineStr">
+      <c r="A38" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor[].affiliation[].name</t>
         </is>
@@ -1620,7 +1647,7 @@
       <c r="M38" s="14" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="18" t="inlineStr">
+      <c r="A39" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor[].affiliation[].affiliation_id</t>
         </is>
@@ -1639,7 +1666,7 @@
       <c r="M39" s="14" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="18" t="inlineStr">
+      <c r="A40" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor[].affiliation[].affiliation_id.identifier</t>
         </is>
@@ -1658,7 +1685,7 @@
       <c r="M40" s="14" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="18" t="inlineStr">
+      <c r="A41" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor[].affiliation[].affiliation_id.type</t>
         </is>
@@ -1677,7 +1704,7 @@
       <c r="M41" s="14" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="18" t="inlineStr">
+      <c r="A42" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor[].role</t>
         </is>
@@ -1696,27 +1723,27 @@
       <c r="M42" s="14" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="18" t="inlineStr">
+      <c r="A43" s="22" t="inlineStr">
         <is>
           <t>dmp.contributor[].role[]</t>
         </is>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B43" s="70" t="inlineStr">
         <is>
           <t>Principal Investigator; Data Manager</t>
         </is>
       </c>
-      <c r="C43" s="22" t="inlineStr">
+      <c r="C43" s="70" t="inlineStr">
         <is>
           <t>Principal Investigator</t>
         </is>
       </c>
-      <c r="D43" s="22" t="inlineStr">
+      <c r="D43" s="70" t="inlineStr">
         <is>
           <t>Data Manager</t>
         </is>
       </c>
-      <c r="E43" s="22" t="inlineStr">
+      <c r="E43" s="70" t="inlineStr">
         <is>
           <t>Data Manager</t>
         </is>
@@ -1731,7 +1758,7 @@
       <c r="M43" s="14" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="18" t="inlineStr">
+      <c r="A44" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset</t>
         </is>
@@ -1750,7 +1777,7 @@
       <c r="M44" s="14" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="18" t="inlineStr">
+      <c r="A45" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[]</t>
         </is>
@@ -1774,57 +1801,57 @@
           <t>dmp.dataset[].title</t>
         </is>
       </c>
-      <c r="B46" s="36" t="inlineStr">
+      <c r="B46" s="70" t="inlineStr">
         <is>
           <t>Hakai Institute Juvenile Salmon Program Time Series</t>
         </is>
       </c>
-      <c r="C46" s="36" t="inlineStr">
+      <c r="C46" s="70" t="inlineStr">
         <is>
           <t>Fatty acids from juvenile salmon</t>
         </is>
       </c>
-      <c r="D46" s="36" t="inlineStr">
+      <c r="D46" s="70" t="inlineStr">
         <is>
           <t>Otolith Microchemistry from juvenile sockeye</t>
         </is>
       </c>
-      <c r="E46" s="36" t="inlineStr">
+      <c r="E46" s="70" t="inlineStr">
         <is>
           <t>Sealice microbiome viral and bacterial data</t>
         </is>
       </c>
-      <c r="F46" s="36" t="inlineStr">
+      <c r="F46" s="70" t="inlineStr">
         <is>
           <t>Stable isotope ratios from juvenile salmon muscle tissue</t>
         </is>
       </c>
-      <c r="G46" s="36" t="inlineStr">
+      <c r="G46" s="70" t="inlineStr">
         <is>
           <t>Zooplankton Isotopes from JSP surface horizontal tows</t>
         </is>
       </c>
-      <c r="H46" s="36" t="inlineStr">
+      <c r="H46" s="70" t="inlineStr">
         <is>
           <t>eDNA from JSP seines</t>
         </is>
       </c>
-      <c r="I46" s="36" t="inlineStr">
+      <c r="I46" s="70" t="inlineStr">
         <is>
           <t>Zooplankton Taxonomy from JSP and Oceanography horizontal surface tows</t>
         </is>
       </c>
-      <c r="J46" s="36" t="inlineStr">
+      <c r="J46" s="70" t="inlineStr">
         <is>
           <t>RNA pathogen and gene expression data: Fitchip data from sockeye</t>
         </is>
       </c>
-      <c r="K46" s="36" t="inlineStr">
+      <c r="K46" s="70" t="inlineStr">
         <is>
           <t>Genetic stock identification of sockeye</t>
         </is>
       </c>
-      <c r="L46" s="36" t="inlineStr">
+      <c r="L46" s="70" t="inlineStr">
         <is>
           <t>Scales collected from sockeye, pink, chum, coho, chinook and herring</t>
         </is>
@@ -1836,62 +1863,62 @@
       <c r="Q46" s="33" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="18" t="inlineStr">
+      <c r="A47" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].type</t>
         </is>
       </c>
-      <c r="B47" s="22" t="inlineStr">
+      <c r="B47" s="70" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="C47" s="22" t="inlineStr">
+      <c r="C47" s="70" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="D47" s="22" t="inlineStr">
+      <c r="D47" s="70" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="E47" s="22" t="inlineStr">
+      <c r="E47" s="70" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="F47" s="22" t="inlineStr">
+      <c r="F47" s="70" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="G47" s="22" t="inlineStr">
+      <c r="G47" s="70" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="H47" s="22" t="inlineStr">
+      <c r="H47" s="70" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="I47" s="22" t="inlineStr">
+      <c r="I47" s="70" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="J47" s="22" t="inlineStr">
+      <c r="J47" s="70" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="K47" s="22" t="inlineStr">
+      <c r="K47" s="70" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="L47" s="22" t="inlineStr">
+      <c r="L47" s="70" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
@@ -1908,57 +1935,57 @@
           <t>dmp.dataset[].description</t>
         </is>
       </c>
-      <c r="B48" s="36" t="inlineStr">
+      <c r="B48" s="70" t="inlineStr">
         <is>
           <t>The core of the Hakai JSP are the observations made at sea during seining operations, and the observations and measurements made in the lab during fish dissections. Many samples are produced from fish that are collected in the lab, and those data may be addressed in their own Data Management Plans.</t>
         </is>
       </c>
-      <c r="C48" s="36" t="inlineStr">
+      <c r="C48" s="70" t="inlineStr">
         <is>
           <t>This dataset will include fatty acid data derived from juvenile salmon tissue samples. Alicia Andersen is going to provide this dataset.</t>
         </is>
       </c>
-      <c r="D48" s="36" t="inlineStr">
+      <c r="D48" s="70" t="inlineStr">
         <is>
           <t>Microchemistry data as obtained from otolith analysis. Otoliths were obtained from juvenile salmon as part of the Juvenile Salmon Program (JSP). The responsible party for this dataset is Yuliya Kuzmenko (UBC). The Paper has been published at https://doi.org/10.26428/1606-9919-2021-201-669-685 but we need to reach out to Yuliya to collect data.</t>
         </is>
       </c>
-      <c r="E48" s="36" t="inlineStr">
+      <c r="E48" s="70" t="inlineStr">
         <is>
           <t>The responsible parties for this dataset are Tianyi Chang and Curtis Suttle. Need an update from Tianyi</t>
         </is>
       </c>
-      <c r="F48" s="36" t="inlineStr">
+      <c r="F48" s="70" t="inlineStr">
         <is>
           <t>This dataset will contain isotope data obtained from juvenile salmon caught during the JSP. The responsible party for this dataset is Brian Hunt.</t>
         </is>
       </c>
-      <c r="G48" s="36" t="inlineStr">
+      <c r="G48" s="70" t="inlineStr">
         <is>
           <t>This dataset will contain isotope data obtained from the zooplankton caught as part of the Juvenile Salmon Program (JSP). Brian Hunt is the responsible party for this dataset.</t>
         </is>
       </c>
-      <c r="H48" s="36" t="inlineStr">
+      <c r="H48" s="70" t="inlineStr">
         <is>
           <t>Environmental DNA (eDNA) is collected as part of the Juvenile Salmon Program field operations, starting in 2020. The responsible party for this dataset is Natalie Benoit (UBC).</t>
         </is>
       </c>
-      <c r="I48" s="36" t="inlineStr">
+      <c r="I48" s="70" t="inlineStr">
         <is>
           <t>An integration of Sam James, Vanessa Fladmark, and Natalie Mahara's zooplankton taxonomy from horizontal surface tows in the Discovery Islands and Johnstone Strait.</t>
         </is>
       </c>
-      <c r="J48" s="36" t="inlineStr">
+      <c r="J48" s="70" t="inlineStr">
         <is>
           <t>Dataset from fish tissue samples sent to Kristi Millers lab. Currently 2015 sockeye, pink and chum dataset is published as part of the Hakai JSP data package. Katherine Medcalf' (UoT) project will produce fit chip data from Krisiti Miller's lab for 2016 sockeye and will be used in conjunction with sea lice count data and the 2015 fit chip data. Katherine is working on a separate DMP for that.</t>
         </is>
       </c>
-      <c r="K48" s="36" t="inlineStr">
+      <c r="K48" s="70" t="inlineStr">
         <is>
           <t>Fin clips and liver samples are sent to the Pacific Biological Station for stock identification. Currently, we have results from 2015–2019. These data could be published in a stand alone data package, with an accompanying data paper. Currently, they reside in the JSP GitHub repo along with the JSP Time-series dataset.</t>
         </is>
       </c>
-      <c r="L48" s="36" t="inlineStr">
+      <c r="L48" s="70" t="inlineStr">
         <is>
           <t>Scales are collected for every salmon and herring and archived. No analysis has been completed at this stage nor is any planned.</t>
         </is>
@@ -1970,7 +1997,7 @@
       <c r="Q48" s="34" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="18" t="inlineStr">
+      <c r="A49" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].dataset_id</t>
         </is>
@@ -1989,12 +2016,12 @@
       <c r="M49" s="14" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="18" t="inlineStr">
+      <c r="A50" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].dataset_id.identifier</t>
         </is>
       </c>
-      <c r="B50" s="27" t="inlineStr">
+      <c r="B50" s="70" t="inlineStr">
         <is>
           <t>https://doi.org/10.21966/1.566666</t>
         </is>
@@ -2012,12 +2039,12 @@
       <c r="M50" s="14" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="18" t="inlineStr">
+      <c r="A51" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].dataset_id.type</t>
         </is>
       </c>
-      <c r="B51" s="22" t="inlineStr">
+      <c r="B51" s="70" t="inlineStr">
         <is>
           <t>doi</t>
         </is>
@@ -2035,62 +2062,62 @@
       <c r="M51" s="14" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="18" t="inlineStr">
+      <c r="A52" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].personal_data</t>
         </is>
       </c>
-      <c r="B52" s="22" t="inlineStr">
+      <c r="B52" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C52" s="22" t="inlineStr">
+      <c r="C52" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="D52" s="22" t="inlineStr">
+      <c r="D52" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="E52" s="22" t="inlineStr">
+      <c r="E52" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="F52" s="22" t="inlineStr">
+      <c r="F52" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="G52" s="22" t="inlineStr">
+      <c r="G52" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H52" s="22" t="inlineStr">
+      <c r="H52" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="I52" s="22" t="inlineStr">
+      <c r="I52" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J52" s="22" t="inlineStr">
+      <c r="J52" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K52" s="22" t="inlineStr">
+      <c r="K52" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="L52" s="22" t="inlineStr">
+      <c r="L52" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2098,62 +2125,62 @@
       <c r="M52" s="14" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="18" t="inlineStr">
+      <c r="A53" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].sensitive_data</t>
         </is>
       </c>
-      <c r="B53" s="22" t="inlineStr">
+      <c r="B53" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C53" s="22" t="inlineStr">
+      <c r="C53" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="D53" s="22" t="inlineStr">
+      <c r="D53" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="E53" s="22" t="inlineStr">
+      <c r="E53" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="F53" s="22" t="inlineStr">
+      <c r="F53" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="G53" s="22" t="inlineStr">
+      <c r="G53" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H53" s="22" t="inlineStr">
+      <c r="H53" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="I53" s="22" t="inlineStr">
+      <c r="I53" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J53" s="22" t="inlineStr">
+      <c r="J53" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K53" s="22" t="inlineStr">
+      <c r="K53" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="L53" s="22" t="inlineStr">
+      <c r="L53" s="70" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2161,7 +2188,7 @@
       <c r="M53" s="14" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="18" t="inlineStr">
+      <c r="A54" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].issued</t>
         </is>
@@ -2180,7 +2207,7 @@
       <c r="M54" s="14" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="18" t="inlineStr">
+      <c r="A55" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].metadata</t>
         </is>
@@ -2199,7 +2226,7 @@
       <c r="M55" s="14" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="18" t="inlineStr">
+      <c r="A56" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].metadata[]</t>
         </is>
@@ -2218,7 +2245,7 @@
       <c r="M56" s="14" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="18" t="inlineStr">
+      <c r="A57" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].metadata[].description</t>
         </is>
@@ -2237,26 +2264,66 @@
       <c r="M57" s="14" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="18" t="inlineStr">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].metadata[].language</t>
         </is>
       </c>
       <c r="B58" s="22" t="n"/>
-      <c r="C58" s="22" t="n"/>
-      <c r="D58" s="22" t="n"/>
-      <c r="E58" s="22" t="n"/>
-      <c r="F58" s="22" t="n"/>
-      <c r="G58" s="22" t="n"/>
-      <c r="H58" s="22" t="n"/>
-      <c r="I58" s="22" t="n"/>
-      <c r="J58" s="22" t="n"/>
-      <c r="K58" s="22" t="n"/>
-      <c r="L58" s="22" t="n"/>
+      <c r="C58" s="70" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="D58" s="70" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="E58" s="70" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="F58" s="70" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="G58" s="70" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="H58" s="70" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="I58" s="70" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="J58" s="70" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="K58" s="70" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="L58" s="70" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
       <c r="M58" s="14" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="18" t="inlineStr">
+      <c r="A59" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].metadata[].metadata_standard_id</t>
         </is>
@@ -2275,7 +2342,7 @@
       <c r="M59" s="14" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="18" t="inlineStr">
+      <c r="A60" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].metadata[].metadata_standard_id[]</t>
         </is>
@@ -2294,26 +2361,26 @@
       <c r="M60" s="14" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="18" t="inlineStr">
+      <c r="A61" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].metadata[].metadata_standard_id[].identifier</t>
         </is>
       </c>
       <c r="B61" s="22" t="n"/>
-      <c r="C61" s="22" t="inlineStr">
+      <c r="C61" s="70" t="inlineStr">
         <is>
           <t>ISO 19115</t>
         </is>
       </c>
       <c r="D61" s="22" t="n"/>
       <c r="E61" s="22" t="n"/>
-      <c r="F61" s="22" t="inlineStr">
+      <c r="F61" s="70" t="inlineStr">
         <is>
           <t>ISO 19115</t>
         </is>
       </c>
       <c r="G61" s="22" t="n"/>
-      <c r="H61" s="22" t="inlineStr">
+      <c r="H61" s="70" t="inlineStr">
         <is>
           <t>ISO 19115 North American Profile; ISO 19115</t>
         </is>
@@ -2325,7 +2392,7 @@
       <c r="M61" s="14" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="18" t="inlineStr">
+      <c r="A62" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].metadata[].metadata_standard_id[].type</t>
         </is>
@@ -2344,7 +2411,7 @@
       <c r="M62" s="14" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="18" t="inlineStr">
+      <c r="A63" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution</t>
         </is>
@@ -2363,7 +2430,7 @@
       <c r="M63" s="14" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="18" t="inlineStr">
+      <c r="A64" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[]</t>
         </is>
@@ -2382,12 +2449,16 @@
       <c r="M64" s="14" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="18" t="inlineStr">
+      <c r="A65" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[].title</t>
         </is>
       </c>
-      <c r="B65" s="22" t="n"/>
+      <c r="B65" s="70" t="inlineStr">
+        <is>
+          <t>Hakai JSP Time Series</t>
+        </is>
+      </c>
       <c r="C65" s="22" t="n"/>
       <c r="D65" s="22" t="n"/>
       <c r="E65" s="22" t="n"/>
@@ -2401,7 +2472,7 @@
       <c r="M65" s="14" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="18" t="inlineStr">
+      <c r="A66" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[].byte_size</t>
         </is>
@@ -2420,7 +2491,7 @@
       <c r="M66" s="14" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="18" t="inlineStr">
+      <c r="A67" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[].issued</t>
         </is>
@@ -2431,11 +2502,15 @@
       <c r="E67" s="22" t="n"/>
       <c r="F67" s="22" t="n"/>
       <c r="G67" s="22" t="n"/>
-      <c r="H67" s="50" t="n">
-        <v>45395</v>
-      </c>
-      <c r="I67" s="50" t="n">
-        <v>44650</v>
+      <c r="H67" s="72" t="inlineStr">
+        <is>
+          <t>2024-04-13</t>
+        </is>
+      </c>
+      <c r="I67" s="72" t="inlineStr">
+        <is>
+          <t>2022-03-30</t>
+        </is>
       </c>
       <c r="J67" s="22" t="n"/>
       <c r="K67" s="22" t="n"/>
@@ -2443,62 +2518,62 @@
       <c r="M67" s="14" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="18" t="inlineStr">
+      <c r="A68" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[].data_access</t>
         </is>
       </c>
-      <c r="B68" s="22" t="inlineStr">
+      <c r="B68" s="70" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="C68" s="22" t="inlineStr">
+      <c r="C68" s="70" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="D68" s="22" t="inlineStr">
+      <c r="D68" s="70" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E68" s="22" t="inlineStr">
+      <c r="E68" s="70" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F68" s="22" t="inlineStr">
+      <c r="F68" s="70" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="G68" s="22" t="inlineStr">
+      <c r="G68" s="70" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="H68" s="22" t="inlineStr">
+      <c r="H68" s="70" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="I68" s="22" t="inlineStr">
+      <c r="I68" s="70" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="J68" s="22" t="inlineStr">
+      <c r="J68" s="70" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="K68" s="22" t="inlineStr">
+      <c r="K68" s="70" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="L68" s="22" t="inlineStr">
+      <c r="L68" s="70" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2506,7 +2581,7 @@
       <c r="M68" s="14" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="18" t="inlineStr">
+      <c r="A69" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[].license</t>
         </is>
@@ -2525,7 +2600,7 @@
       <c r="M69" s="14" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="18" t="inlineStr">
+      <c r="A70" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[].license[]</t>
         </is>
@@ -2544,52 +2619,52 @@
       <c r="M70" s="14" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="18" t="inlineStr">
+      <c r="A71" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[].license[].license_ref</t>
         </is>
       </c>
-      <c r="B71" s="22" t="inlineStr">
+      <c r="B71" s="70" t="inlineStr">
         <is>
           <t>CC BY 4.0</t>
         </is>
       </c>
-      <c r="C71" s="22" t="inlineStr">
+      <c r="C71" s="70" t="inlineStr">
         <is>
           <t>CC BY 4.0</t>
         </is>
       </c>
-      <c r="D71" s="22" t="inlineStr">
+      <c r="D71" s="70" t="inlineStr">
         <is>
           <t>CC BY 4.0</t>
         </is>
       </c>
-      <c r="E71" s="22" t="inlineStr">
+      <c r="E71" s="70" t="inlineStr">
         <is>
           <t>CC BY 4.0</t>
         </is>
       </c>
-      <c r="F71" s="22" t="inlineStr">
+      <c r="F71" s="70" t="inlineStr">
         <is>
           <t>CC BY 4.0</t>
         </is>
       </c>
-      <c r="G71" s="22" t="inlineStr">
+      <c r="G71" s="70" t="inlineStr">
         <is>
           <t>CC BY 4.0</t>
         </is>
       </c>
-      <c r="H71" s="22" t="inlineStr">
+      <c r="H71" s="70" t="inlineStr">
         <is>
           <t>CC BY 4.0</t>
         </is>
       </c>
-      <c r="I71" s="22" t="inlineStr">
+      <c r="I71" s="70" t="inlineStr">
         <is>
           <t>CC BY 4.0</t>
         </is>
       </c>
-      <c r="J71" s="22" t="inlineStr">
+      <c r="J71" s="70" t="inlineStr">
         <is>
           <t>CC BY 4.0</t>
         </is>
@@ -2599,7 +2674,7 @@
       <c r="M71" s="14" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="18" t="inlineStr">
+      <c r="A72" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[].license[].start_date</t>
         </is>
@@ -2618,7 +2693,7 @@
       <c r="M72" s="14" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="18" t="inlineStr">
+      <c r="A73" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[].host</t>
         </is>
@@ -2642,49 +2717,53 @@
           <t>dmp.dataset[].distribution[].host.title</t>
         </is>
       </c>
-      <c r="B74" s="36" t="inlineStr">
+      <c r="B74" s="70" t="inlineStr">
         <is>
           <t>Hakai JSP GitHub repository</t>
         </is>
       </c>
-      <c r="C74" s="36" t="inlineStr">
+      <c r="C74" s="70" t="inlineStr">
         <is>
           <t>Hakai EIMS</t>
         </is>
       </c>
-      <c r="D74" s="36" t="inlineStr">
+      <c r="D74" s="70" t="inlineStr">
         <is>
           <t>Hakai EIMS</t>
         </is>
       </c>
       <c r="E74" s="36" t="n"/>
-      <c r="F74" s="36" t="inlineStr">
+      <c r="F74" s="70" t="inlineStr">
         <is>
           <t>Hakai EIMS</t>
         </is>
       </c>
       <c r="G74" s="36" t="n"/>
-      <c r="H74" s="36" t="inlineStr">
+      <c r="H74" s="70" t="inlineStr">
         <is>
           <t>Ocean Biodiversity Information System</t>
         </is>
       </c>
-      <c r="I74" s="36" t="inlineStr">
+      <c r="I74" s="70" t="inlineStr">
         <is>
           <t>Hakai EIMS; Ocean Biogeographic Information System</t>
         </is>
       </c>
-      <c r="J74" s="36" t="inlineStr">
+      <c r="J74" s="70" t="inlineStr">
         <is>
           <t>Hakai EIMS</t>
         </is>
       </c>
-      <c r="K74" s="36" t="inlineStr">
+      <c r="K74" s="70" t="inlineStr">
         <is>
           <t>Ocean Biogeographic Information System</t>
         </is>
       </c>
-      <c r="L74" s="36" t="n"/>
+      <c r="L74" s="70" t="inlineStr">
+        <is>
+          <t>Ocean Biogeographic Information System</t>
+        </is>
+      </c>
       <c r="M74" s="32" t="n"/>
       <c r="N74" s="33" t="n"/>
       <c r="O74" s="33" t="n"/>
@@ -2692,12 +2771,12 @@
       <c r="Q74" s="33" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="18" t="inlineStr">
+      <c r="A75" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[].host.url</t>
         </is>
       </c>
-      <c r="B75" s="27" t="inlineStr">
+      <c r="B75" s="70" t="inlineStr">
         <is>
           <t>https://github.com/hakaiinstitute/jsp-data</t>
         </is>
@@ -2715,7 +2794,7 @@
       <c r="M75" s="14" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="18" t="inlineStr">
+      <c r="A76" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[].host.host_id</t>
         </is>
@@ -2734,7 +2813,7 @@
       <c r="M76" s="14" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="18" t="inlineStr">
+      <c r="A77" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[].host.host_id[]</t>
         </is>
@@ -2753,7 +2832,7 @@
       <c r="M77" s="14" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="18" t="inlineStr">
+      <c r="A78" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[].host.host_id[].identifier</t>
         </is>
@@ -2772,7 +2851,7 @@
       <c r="M78" s="14" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="18" t="inlineStr">
+      <c r="A79" s="22" t="inlineStr">
         <is>
           <t>dmp.dataset[].distribution[].host.host_id[].type</t>
         </is>
@@ -2791,7 +2870,7 @@
       <c r="M79" s="14" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="18" t="inlineStr">
+      <c r="A80" s="22" t="inlineStr">
         <is>
           <t>dmp.related_identifier</t>
         </is>
@@ -2810,7 +2889,7 @@
       <c r="M80" s="14" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="18" t="inlineStr">
+      <c r="A81" s="22" t="inlineStr">
         <is>
           <t>dmp.related_identifier[]</t>
         </is>
@@ -2829,12 +2908,12 @@
       <c r="M81" s="14" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="18" t="inlineStr">
+      <c r="A82" s="22" t="inlineStr">
         <is>
           <t>dmp.related_identifier[].identifier</t>
         </is>
       </c>
-      <c r="B82" s="27" t="inlineStr">
+      <c r="B82" s="70" t="inlineStr">
         <is>
           <t>https://doi.org/10.26428/1606-9919-2021-201-669-685</t>
         </is>
@@ -2852,7 +2931,7 @@
       <c r="M82" s="14" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="18" t="inlineStr">
+      <c r="A83" s="22" t="inlineStr">
         <is>
           <t>dmp.related_identifier[].relation_type</t>
         </is>
@@ -2871,7 +2950,7 @@
       <c r="M83" s="14" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="18" t="inlineStr">
+      <c r="A84" s="22" t="inlineStr">
         <is>
           <t>dmp.related_identifier[].resource_type</t>
         </is>
@@ -2890,7 +2969,7 @@
       <c r="M84" s="14" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="18" t="inlineStr">
+      <c r="A85" s="22" t="inlineStr">
         <is>
           <t>dmp.related_identifier[].type</t>
         </is>
@@ -2909,7 +2988,7 @@
       <c r="M85" s="14" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="18" t="inlineStr">
+      <c r="A86" s="22" t="inlineStr">
         <is>
           <t>dmp.alternate_identifier</t>
         </is>
@@ -2928,7 +3007,7 @@
       <c r="M86" s="14" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="18" t="inlineStr">
+      <c r="A87" s="22" t="inlineStr">
         <is>
           <t>dmp.alternate_identifier[]</t>
         </is>
@@ -2947,7 +3026,7 @@
       <c r="M87" s="14" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="18" t="inlineStr">
+      <c r="A88" s="22" t="inlineStr">
         <is>
           <t>dmp.alternate_identifier[].identifier</t>
         </is>
@@ -2966,7 +3045,7 @@
       <c r="M88" s="14" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="18" t="inlineStr">
+      <c r="A89" s="22" t="inlineStr">
         <is>
           <t>dmp.alternate_identifier[].type</t>
         </is>
@@ -2985,7 +3064,7 @@
       <c r="M89" s="14" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="18" t="inlineStr">
+      <c r="A90" s="22" t="inlineStr">
         <is>
           <t>dmp.project</t>
         </is>
@@ -3004,7 +3083,7 @@
       <c r="M90" s="14" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="18" t="inlineStr">
+      <c r="A91" s="22" t="inlineStr">
         <is>
           <t>dmp.project[]</t>
         </is>
@@ -3023,12 +3102,16 @@
       <c r="M91" s="14" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="18" t="inlineStr">
+      <c r="A92" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].title</t>
         </is>
       </c>
-      <c r="B92" s="22" t="n"/>
+      <c r="B92" s="70" t="inlineStr">
+        <is>
+          <t>Hakai JSP Time Series</t>
+        </is>
+      </c>
       <c r="C92" s="22" t="n"/>
       <c r="D92" s="22" t="n"/>
       <c r="E92" s="22" t="n"/>
@@ -3047,7 +3130,7 @@
           <t>dmp.project[].description</t>
         </is>
       </c>
-      <c r="B93" s="36" t="inlineStr">
+      <c r="B93" s="70" t="inlineStr">
         <is>
           <t>The Hakai Institute Juvenile Salmon program is an ongoing initiative that was established in 2015 in partnership with the University of British Columbia, University of Toronto, Simon Fraser University and Salmon Coast Field Station. This program researches the early life history of juvenile salmon in coastal British Columbia. Primary research objectives are determining: 1) Migration timing rates and routes; 2) Migration habitat, including physical and chemical oceanographic conditions, and availability of plankton prey; 3) The impacts of prey phenology, quantity and quality on juvenile salmon growth and condition; 4) Species and stock-specific feeding biology and competitive interactions; 5) Pathogen and parasite infection dynamics; and 6) Mortality estimates. The program targets Fraser River sockeye, and pink and chum salmon, but additionally provides information on coho, chinook, and herring through incidental capture. The field program operates between May and July during the peak of the juvenile sockeye outward migration. Purse seine and oceanographic sampling are conducted in the northern Strait of Georgia / Discovery Islands region (~ 220 km from the Fraser River mouth).</t>
         </is>
@@ -3069,7 +3152,7 @@
       <c r="Q93" s="33" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="18" t="inlineStr">
+      <c r="A94" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].project_id</t>
         </is>
@@ -3088,7 +3171,7 @@
       <c r="M94" s="14" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="18" t="inlineStr">
+      <c r="A95" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].project_id[]</t>
         </is>
@@ -3107,7 +3190,7 @@
       <c r="M95" s="14" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="18" t="inlineStr">
+      <c r="A96" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].project_id[].identifier</t>
         </is>
@@ -3126,7 +3209,7 @@
       <c r="M96" s="14" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="18" t="inlineStr">
+      <c r="A97" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].project_id[].type</t>
         </is>
@@ -3145,13 +3228,15 @@
       <c r="M97" s="14" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="18" t="inlineStr">
+      <c r="A98" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].start</t>
         </is>
       </c>
-      <c r="B98" s="50" t="n">
-        <v>42136</v>
+      <c r="B98" s="72" t="inlineStr">
+        <is>
+          <t>2015-05-12</t>
+        </is>
       </c>
       <c r="C98" s="22" t="n"/>
       <c r="D98" s="22" t="n"/>
@@ -3166,13 +3251,15 @@
       <c r="M98" s="14" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="18" t="inlineStr">
+      <c r="A99" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].end</t>
         </is>
       </c>
-      <c r="B99" s="50" t="n">
-        <v>45112</v>
+      <c r="B99" s="72" t="inlineStr">
+        <is>
+          <t>2023-07-05</t>
+        </is>
       </c>
       <c r="C99" s="22" t="n"/>
       <c r="D99" s="22" t="n"/>
@@ -3187,7 +3274,7 @@
       <c r="M99" s="14" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="18" t="inlineStr">
+      <c r="A100" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].funding</t>
         </is>
@@ -3206,7 +3293,7 @@
       <c r="M100" s="14" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="18" t="inlineStr">
+      <c r="A101" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].funding[]</t>
         </is>
@@ -3225,12 +3312,12 @@
       <c r="M101" s="14" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="18" t="inlineStr">
+      <c r="A102" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].funding[].name</t>
         </is>
       </c>
-      <c r="B102" s="22" t="inlineStr">
+      <c r="B102" s="70" t="inlineStr">
         <is>
           <t>Tula Foundation</t>
         </is>
@@ -3248,7 +3335,7 @@
       <c r="M102" s="14" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="18" t="inlineStr">
+      <c r="A103" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].funding[].funding_status</t>
         </is>
@@ -3267,7 +3354,7 @@
       <c r="M103" s="14" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="18" t="inlineStr">
+      <c r="A104" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].funding[].funder_id</t>
         </is>
@@ -3286,7 +3373,7 @@
       <c r="M104" s="14" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="18" t="inlineStr">
+      <c r="A105" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].funding[].funder_id.identifier</t>
         </is>
@@ -3305,7 +3392,7 @@
       <c r="M105" s="14" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="18" t="inlineStr">
+      <c r="A106" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].funding[].funder_id.type</t>
         </is>
@@ -3324,7 +3411,7 @@
       <c r="M106" s="14" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="18" t="inlineStr">
+      <c r="A107" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].funding[].grant_id</t>
         </is>
@@ -3343,7 +3430,7 @@
       <c r="M107" s="14" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="18" t="inlineStr">
+      <c r="A108" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].funding[].grant_id[]</t>
         </is>
@@ -3362,7 +3449,7 @@
       <c r="M108" s="14" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="18" t="inlineStr">
+      <c r="A109" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].funding[].grant_id[].identifier</t>
         </is>
@@ -3381,7 +3468,7 @@
       <c r="M109" s="14" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="18" t="inlineStr">
+      <c r="A110" s="22" t="inlineStr">
         <is>
           <t>dmp.project[].funding[].grant_id[].type</t>
         </is>
@@ -3400,7 +3487,7 @@
       <c r="M110" s="14" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="18" t="inlineStr">
+      <c r="A111" s="22" t="inlineStr">
         <is>
           <t>rda_schema_version</t>
         </is>
@@ -3419,7 +3506,7 @@
       <c r="M111" s="14" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="18" t="inlineStr">
+      <c r="A112" s="22" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
@@ -3438,7 +3525,7 @@
       <c r="M112" s="14" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="18" t="inlineStr">
+      <c r="A113" s="22" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -3457,7 +3544,7 @@
       <c r="M113" s="14" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="18" t="inlineStr">
+      <c r="A114" s="22" t="inlineStr">
         <is>
           <t>privacy</t>
         </is>
@@ -3476,7 +3563,7 @@
       <c r="M114" s="14" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="18" t="inlineStr">
+      <c r="A115" s="22" t="inlineStr">
         <is>
           <t>featured</t>
         </is>
@@ -3495,7 +3582,7 @@
       <c r="M115" s="14" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="18" t="inlineStr">
+      <c r="A116" s="22" t="inlineStr">
         <is>
           <t>registered</t>
         </is>
@@ -3514,7 +3601,7 @@
       <c r="M116" s="14" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="18" t="inlineStr">
+      <c r="A117" s="22" t="inlineStr">
         <is>
           <t>research_domain</t>
         </is>
@@ -3552,7 +3639,7 @@
       <c r="M118" s="14" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="18" t="inlineStr">
+      <c r="A119" s="22" t="inlineStr">
         <is>
           <t>research_domain.research_domain_identifier</t>
         </is>
@@ -3571,7 +3658,7 @@
       <c r="M119" s="14" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="18" t="inlineStr">
+      <c r="A120" s="22" t="inlineStr">
         <is>
           <t>research_domain.research_domain_identifier.identifier</t>
         </is>
@@ -3590,7 +3677,7 @@
       <c r="M120" s="14" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="18" t="inlineStr">
+      <c r="A121" s="22" t="inlineStr">
         <is>
           <t>research_domain.research_domain_identifier.type</t>
         </is>
@@ -3609,7 +3696,7 @@
       <c r="M121" s="14" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="18" t="inlineStr">
+      <c r="A122" s="22" t="inlineStr">
         <is>
           <t>research_facility</t>
         </is>
@@ -3628,7 +3715,7 @@
       <c r="M122" s="14" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="18" t="inlineStr">
+      <c r="A123" s="22" t="inlineStr">
         <is>
           <t>research_facility[]</t>
         </is>
@@ -3647,7 +3734,7 @@
       <c r="M123" s="14" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="18" t="inlineStr">
+      <c r="A124" s="22" t="inlineStr">
         <is>
           <t>research_facility[].name</t>
         </is>
@@ -3666,7 +3753,7 @@
       <c r="M124" s="14" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" s="18" t="inlineStr">
+      <c r="A125" s="22" t="inlineStr">
         <is>
           <t>research_facility[].type</t>
         </is>
@@ -3685,7 +3772,7 @@
       <c r="M125" s="14" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="18" t="inlineStr">
+      <c r="A126" s="22" t="inlineStr">
         <is>
           <t>research_facility[].research_facility_identifier</t>
         </is>
@@ -3704,7 +3791,7 @@
       <c r="M126" s="14" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="18" t="inlineStr">
+      <c r="A127" s="22" t="inlineStr">
         <is>
           <t>research_facility[].research_facility_identifier.identifier</t>
         </is>
@@ -3723,7 +3810,7 @@
       <c r="M127" s="14" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="18" t="inlineStr">
+      <c r="A128" s="22" t="inlineStr">
         <is>
           <t>research_facility[].research_facility_identifier.type</t>
         </is>
@@ -3742,7 +3829,7 @@
       <c r="M128" s="14" t="n"/>
     </row>
     <row r="129">
-      <c r="A129" s="18" t="inlineStr">
+      <c r="A129" s="22" t="inlineStr">
         <is>
           <t>funding_opportunity</t>
         </is>
@@ -3761,7 +3848,7 @@
       <c r="M129" s="14" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="18" t="inlineStr">
+      <c r="A130" s="22" t="inlineStr">
         <is>
           <t>funding_opportunity[]</t>
         </is>
@@ -3780,7 +3867,7 @@
       <c r="M130" s="14" t="n"/>
     </row>
     <row r="131">
-      <c r="A131" s="18" t="inlineStr">
+      <c r="A131" s="22" t="inlineStr">
         <is>
           <t>funding_opportunity[].project_id</t>
         </is>
@@ -3799,7 +3886,7 @@
       <c r="M131" s="14" t="n"/>
     </row>
     <row r="132">
-      <c r="A132" s="18" t="inlineStr">
+      <c r="A132" s="22" t="inlineStr">
         <is>
           <t>funding_opportunity[].project_id.identifier</t>
         </is>
@@ -3818,7 +3905,7 @@
       <c r="M132" s="14" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="18" t="inlineStr">
+      <c r="A133" s="22" t="inlineStr">
         <is>
           <t>funding_opportunity[].project_id.type</t>
         </is>
@@ -3837,7 +3924,7 @@
       <c r="M133" s="14" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="18" t="inlineStr">
+      <c r="A134" s="22" t="inlineStr">
         <is>
           <t>funding_opportunity[].funder_id</t>
         </is>
@@ -3856,7 +3943,7 @@
       <c r="M134" s="14" t="n"/>
     </row>
     <row r="135">
-      <c r="A135" s="18" t="inlineStr">
+      <c r="A135" s="22" t="inlineStr">
         <is>
           <t>funding_opportunity[].funder_id.identifier</t>
         </is>
@@ -3875,7 +3962,7 @@
       <c r="M135" s="14" t="n"/>
     </row>
     <row r="136">
-      <c r="A136" s="18" t="inlineStr">
+      <c r="A136" s="22" t="inlineStr">
         <is>
           <t>funding_opportunity[].funder_id.type</t>
         </is>
@@ -3894,7 +3981,7 @@
       <c r="M136" s="14" t="n"/>
     </row>
     <row r="137">
-      <c r="A137" s="18" t="inlineStr">
+      <c r="A137" s="22" t="inlineStr">
         <is>
           <t>funding_opportunity[].opportunity_identifier</t>
         </is>
@@ -3913,7 +4000,7 @@
       <c r="M137" s="14" t="n"/>
     </row>
     <row r="138">
-      <c r="A138" s="18" t="inlineStr">
+      <c r="A138" s="22" t="inlineStr">
         <is>
           <t>funding_opportunity[].opportunity_identifier.identifier</t>
         </is>
@@ -3932,7 +4019,7 @@
       <c r="M138" s="14" t="n"/>
     </row>
     <row r="139">
-      <c r="A139" s="18" t="inlineStr">
+      <c r="A139" s="22" t="inlineStr">
         <is>
           <t>funding_opportunity[].opportunity_identifier.type</t>
         </is>
@@ -3951,7 +4038,7 @@
       <c r="M139" s="14" t="n"/>
     </row>
     <row r="140">
-      <c r="A140" s="18" t="inlineStr">
+      <c r="A140" s="22" t="inlineStr">
         <is>
           <t>funding_project</t>
         </is>
@@ -3970,7 +4057,7 @@
       <c r="M140" s="14" t="n"/>
     </row>
     <row r="141">
-      <c r="A141" s="18" t="inlineStr">
+      <c r="A141" s="22" t="inlineStr">
         <is>
           <t>funding_project[]</t>
         </is>
@@ -3989,7 +4076,7 @@
       <c r="M141" s="14" t="n"/>
     </row>
     <row r="142">
-      <c r="A142" s="18" t="inlineStr">
+      <c r="A142" s="22" t="inlineStr">
         <is>
           <t>funding_project[].project_id</t>
         </is>
@@ -4008,7 +4095,7 @@
       <c r="M142" s="14" t="n"/>
     </row>
     <row r="143">
-      <c r="A143" s="18" t="inlineStr">
+      <c r="A143" s="22" t="inlineStr">
         <is>
           <t>funding_project[].project_id.identifier</t>
         </is>
@@ -4027,7 +4114,7 @@
       <c r="M143" s="14" t="n"/>
     </row>
     <row r="144">
-      <c r="A144" s="18" t="inlineStr">
+      <c r="A144" s="22" t="inlineStr">
         <is>
           <t>funding_project[].project_id.type</t>
         </is>
@@ -4046,7 +4133,7 @@
       <c r="M144" s="14" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="18" t="inlineStr">
+      <c r="A145" s="22" t="inlineStr">
         <is>
           <t>funding_project[].funder_id</t>
         </is>
@@ -4065,7 +4152,7 @@
       <c r="M145" s="14" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="18" t="inlineStr">
+      <c r="A146" s="22" t="inlineStr">
         <is>
           <t>funding_project[].funder_id.identifier</t>
         </is>
@@ -4084,7 +4171,7 @@
       <c r="M146" s="14" t="n"/>
     </row>
     <row r="147">
-      <c r="A147" s="18" t="inlineStr">
+      <c r="A147" s="22" t="inlineStr">
         <is>
           <t>funding_project[].funder_id.type</t>
         </is>
@@ -4103,7 +4190,7 @@
       <c r="M147" s="14" t="n"/>
     </row>
     <row r="148">
-      <c r="A148" s="18" t="inlineStr">
+      <c r="A148" s="22" t="inlineStr">
         <is>
           <t>funding_project[].project_identifier</t>
         </is>
@@ -4122,7 +4209,7 @@
       <c r="M148" s="14" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="18" t="inlineStr">
+      <c r="A149" s="22" t="inlineStr">
         <is>
           <t>funding_project[].project_identifier.identifier</t>
         </is>
@@ -4141,7 +4228,7 @@
       <c r="M149" s="14" t="n"/>
     </row>
     <row r="150">
-      <c r="A150" s="18" t="inlineStr">
+      <c r="A150" s="22" t="inlineStr">
         <is>
           <t>funding_project[].project_identifier.type</t>
         </is>
@@ -4160,7 +4247,7 @@
       <c r="M150" s="14" t="n"/>
     </row>
     <row r="151">
-      <c r="A151" s="18" t="inlineStr">
+      <c r="A151" s="22" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -4179,7 +4266,7 @@
       <c r="M151" s="14" t="n"/>
     </row>
     <row r="152">
-      <c r="A152" s="18" t="inlineStr">
+      <c r="A152" s="22" t="inlineStr">
         <is>
           <t>version[]</t>
         </is>
@@ -4198,7 +4285,7 @@
       <c r="M152" s="14" t="n"/>
     </row>
     <row r="153">
-      <c r="A153" s="18" t="inlineStr">
+      <c r="A153" s="22" t="inlineStr">
         <is>
           <t>version[].access_url</t>
         </is>
@@ -4217,7 +4304,7 @@
       <c r="M153" s="14" t="n"/>
     </row>
     <row r="154">
-      <c r="A154" s="18" t="inlineStr">
+      <c r="A154" s="22" t="inlineStr">
         <is>
           <t>version[].version</t>
         </is>
@@ -4239,13 +4326,21 @@
       <c r="A155" s="51" t="n"/>
     </row>
     <row r="156">
-      <c r="A156" s="51" t="n"/>
+      <c r="A156" s="73" t="inlineStr">
+        <is>
+          <t>Regenerated from RDA_DMP_sample14_manual_annotation.json on 2026-10-02: 134 values. Item k = the k-th dataset / contributor; lists nested below that are joined with '; '.</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="51" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="51" t="n"/>
+      <c r="A158" s="73" t="inlineStr">
+        <is>
+          <t>Regenerated from RDA_DMP_sample14_manual_annotation.json on 2026-10-02: 134 values. Item k = the k-th dataset / contributor; lists nested below that are joined with '; '.</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="51" t="n"/>

</xml_diff>